<commit_message>
Add signal morphology validation + update results
- validate_segments.py: ECG/SCG morphological validity checks
  - ECG: R-peak prominence + autocorrelation HR + QRS width + SNR
  - SCG: Hilbert envelope periodicity + mouse HR range + SNR
- Filtered: ECG 286/315 (90.8%), SCG 276/315 (87.6%)
- Final dataset: 255 ECG + 276 SCG segments
- Updated README with honest results after signal validation

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labels_for_ecg.xlsx
+++ b/labels_for_ecg.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B316"/>
+  <dimension ref="A1:B256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>4_29_T372_seg0.csv</t>
+          <t>4_29_T373_seg0.csv</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -451,27 +451,27 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>4_29_T373_seg0.csv</t>
+          <t>4_29_T374_seg0.csv</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>4_29_T374_seg0.csv</t>
+          <t>4_29_T511_seg0.csv</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>4_29_T377_seg0.csv</t>
+          <t>4_29_T514_seg0.csv</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -481,7 +481,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>4_29_T503_seg4.csv</t>
+          <t>4_29_T516_seg0.csv</t>
         </is>
       </c>
       <c r="B7" t="n">
@@ -491,7 +491,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>4_29_T508_seg0.csv</t>
+          <t>4_29_T517_seg0.csv</t>
         </is>
       </c>
       <c r="B8" t="n">
@@ -501,7 +501,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>4_29_T511_seg0.csv</t>
+          <t>4_29_T518_seg0.csv</t>
         </is>
       </c>
       <c r="B9" t="n">
@@ -511,7 +511,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>4_29_T514_seg0.csv</t>
+          <t>4_29_T520_seg0.csv</t>
         </is>
       </c>
       <c r="B10" t="n">
@@ -521,7 +521,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>4_29_T515_seg0.csv</t>
+          <t>4_30_T418_seg0.csv</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -531,7 +531,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>4_29_T516_seg0.csv</t>
+          <t>4_30_T427_seg0.csv</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -541,7 +541,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>4_29_T517_seg0.csv</t>
+          <t>4_30_T428_seg0.csv</t>
         </is>
       </c>
       <c r="B13" t="n">
@@ -551,7 +551,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>4_29_T518_seg0.csv</t>
+          <t>4_30_T431_seg0.csv</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -561,7 +561,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4_29_T519_seg0.csv</t>
+          <t>4_30_T432_seg0.csv</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -571,7 +571,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>4_29_T520_seg0.csv</t>
+          <t>4_30_T433_seg0.csv</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -581,7 +581,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4_30_T366_seg18.csv</t>
+          <t>4_30_T436_seg0.csv</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -591,7 +591,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>4_30_T418_seg0.csv</t>
+          <t>4_30_T437_seg0.csv</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -601,7 +601,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4_30_T427_seg0.csv</t>
+          <t>5_14_T357_seg0.csv</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -611,7 +611,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>4_30_T428_seg0.csv</t>
+          <t>5_14_T359_seg0.csv</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -621,7 +621,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>4_30_T431_seg0.csv</t>
+          <t>5_14_T373_seg0.csv</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -631,17 +631,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>4_30_T432_seg0.csv</t>
+          <t>5_14_T376_seg0.csv</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>4_30_T433_seg0.csv</t>
+          <t>5_14_T377_seg9.csv</t>
         </is>
       </c>
       <c r="B23" t="n">
@@ -651,17 +651,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>4_30_T436_seg0.csv</t>
+          <t>5_14_T416_seg11.csv</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>4_30_T437_seg0.csv</t>
+          <t>5_14_T422_seg0.csv</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -671,7 +671,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>5_14_T356_seg0.csv</t>
+          <t>5_14_T424_seg0.csv</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -681,7 +681,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>5_14_T357_seg0.csv</t>
+          <t>5_14_T425_seg0.csv</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -691,7 +691,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>5_14_T358_seg0.csv</t>
+          <t>5_14_T426_seg0.csv</t>
         </is>
       </c>
       <c r="B28" t="n">
@@ -701,7 +701,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>5_14_T359_seg0.csv</t>
+          <t>5_14_T427_seg0.csv</t>
         </is>
       </c>
       <c r="B29" t="n">
@@ -711,7 +711,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5_14_T373_seg0.csv</t>
+          <t>5_14_T429_seg3.csv</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -721,17 +721,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>5_14_T376_seg0.csv</t>
+          <t>5_14_T431_seg0.csv</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>5_14_T377_seg9.csv</t>
+          <t>5_14_T432_seg0.csv</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -741,17 +741,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5_14_T416_seg11.csv</t>
+          <t>5_14_T434_seg0.csv</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>5_14_T422_seg0.csv</t>
+          <t>5_14_T436_seg0.csv</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -761,7 +761,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>5_14_T424_seg0.csv</t>
+          <t>5_14_T438_seg0.csv</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -771,7 +771,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5_14_T425_seg0.csv</t>
+          <t>5_14_T439_seg0.csv</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -781,7 +781,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>5_14_T426_seg0.csv</t>
+          <t>5_14_T440_seg0.csv</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -791,7 +791,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>5_14_T427_seg0.csv</t>
+          <t>5_14_T444_seg0.csv</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -801,7 +801,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>5_14_T428_seg0.csv</t>
+          <t>5_14_T445_seg0.csv</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -811,7 +811,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>5_14_T429_seg3.csv</t>
+          <t>5_14_T447_seg0.csv</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -821,7 +821,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>5_14_T431_seg0.csv</t>
+          <t>5_14_T448_seg0.csv</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -831,7 +831,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>5_14_T432_seg0.csv</t>
+          <t>5_14_T449_seg0.csv</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -841,7 +841,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>5_14_T434_seg0.csv</t>
+          <t>5_14_T450_seg15.csv</t>
         </is>
       </c>
       <c r="B43" t="n">
@@ -851,7 +851,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>5_14_T436_seg0.csv</t>
+          <t>5_14_T451_seg0.csv</t>
         </is>
       </c>
       <c r="B44" t="n">
@@ -861,7 +861,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>5_14_T438_seg0.csv</t>
+          <t>5_14_T452_seg0.csv</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -871,7 +871,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5_14_T439_seg0.csv</t>
+          <t>5_14_T454_seg0.csv</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -881,7 +881,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>5_14_T440_seg0.csv</t>
+          <t>5_14_T455_seg3.csv</t>
         </is>
       </c>
       <c r="B47" t="n">
@@ -891,7 +891,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>5_14_T444_seg0.csv</t>
+          <t>5_14_T457_seg0.csv</t>
         </is>
       </c>
       <c r="B48" t="n">
@@ -901,7 +901,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>5_14_T445_seg0.csv</t>
+          <t>5_14_T458_seg0.csv</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -911,7 +911,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>5_14_T447_seg0.csv</t>
+          <t>5_14_T460_seg0.csv</t>
         </is>
       </c>
       <c r="B50" t="n">
@@ -921,7 +921,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>5_14_T448_seg0.csv</t>
+          <t>5_14_T481_seg0.csv</t>
         </is>
       </c>
       <c r="B51" t="n">
@@ -931,7 +931,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>5_14_T449_seg0.csv</t>
+          <t>5_14_T484_seg1.csv</t>
         </is>
       </c>
       <c r="B52" t="n">
@@ -941,7 +941,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>5_14_T450_seg15.csv</t>
+          <t>5_14_T486_seg0.csv</t>
         </is>
       </c>
       <c r="B53" t="n">
@@ -951,7 +951,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>5_14_T451_seg0.csv</t>
+          <t>5_14_T488_seg0.csv</t>
         </is>
       </c>
       <c r="B54" t="n">
@@ -961,7 +961,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>5_14_T452_seg0.csv</t>
+          <t>5_14_T503_seg2.csv</t>
         </is>
       </c>
       <c r="B55" t="n">
@@ -971,7 +971,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>5_14_T453_seg1.csv</t>
+          <t>5_14_T511_seg0.csv</t>
         </is>
       </c>
       <c r="B56" t="n">
@@ -981,7 +981,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>5_14_T454_seg0.csv</t>
+          <t>5_14_T512_seg15.csv</t>
         </is>
       </c>
       <c r="B57" t="n">
@@ -991,7 +991,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>5_14_T455_seg3.csv</t>
+          <t>5_14_T513_seg0.csv</t>
         </is>
       </c>
       <c r="B58" t="n">
@@ -1001,7 +1001,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>5_14_T456_seg0.csv</t>
+          <t>5_14_T514_seg0.csv</t>
         </is>
       </c>
       <c r="B59" t="n">
@@ -1011,7 +1011,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>5_14_T457_seg0.csv</t>
+          <t>5_14_T517_seg0.csv</t>
         </is>
       </c>
       <c r="B60" t="n">
@@ -1021,7 +1021,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>5_14_T458_seg0.csv</t>
+          <t>5_14_T519_seg0.csv</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -1031,7 +1031,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>5_14_T459_seg0.csv</t>
+          <t>5_28_T366_seg0.csv</t>
         </is>
       </c>
       <c r="B62" t="n">
@@ -1041,7 +1041,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>5_14_T460_seg0.csv</t>
+          <t>5_28_T372_seg0.csv</t>
         </is>
       </c>
       <c r="B63" t="n">
@@ -1051,7 +1051,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>5_14_T481_seg0.csv</t>
+          <t>5_28_T416_seg7.csv</t>
         </is>
       </c>
       <c r="B64" t="n">
@@ -1061,7 +1061,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>5_14_T482_seg0.csv</t>
+          <t>5_28_T418_seg0.csv</t>
         </is>
       </c>
       <c r="B65" t="n">
@@ -1071,17 +1071,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>5_14_T483_seg0.csv</t>
+          <t>5_28_T419_seg20.csv</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>5_14_T484_seg1.csv</t>
+          <t>5_28_T420_seg7.csv</t>
         </is>
       </c>
       <c r="B67" t="n">
@@ -1091,7 +1091,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>5_14_T485_seg0.csv</t>
+          <t>5_28_T421_seg0.csv</t>
         </is>
       </c>
       <c r="B68" t="n">
@@ -1101,7 +1101,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>5_14_T486_seg0.csv</t>
+          <t>5_28_T422_seg0.csv</t>
         </is>
       </c>
       <c r="B69" t="n">
@@ -1111,7 +1111,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>5_14_T487_seg0.csv</t>
+          <t>5_28_T423_seg0.csv</t>
         </is>
       </c>
       <c r="B70" t="n">
@@ -1121,7 +1121,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>5_14_T488_seg0.csv</t>
+          <t>5_28_T424_seg0.csv</t>
         </is>
       </c>
       <c r="B71" t="n">
@@ -1131,7 +1131,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>5_14_T503_seg2.csv</t>
+          <t>5_28_T425_seg0.csv</t>
         </is>
       </c>
       <c r="B72" t="n">
@@ -1141,27 +1141,27 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>5_14_T509_seg3.csv</t>
+          <t>5_28_T427_seg0.csv</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>5_14_T511_seg0.csv</t>
+          <t>5_28_T430_seg0.csv</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>5_14_T512_seg15.csv</t>
+          <t>5_28_T431_seg0.csv</t>
         </is>
       </c>
       <c r="B75" t="n">
@@ -1171,7 +1171,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>5_14_T513_seg0.csv</t>
+          <t>5_28_T435_seg0.csv</t>
         </is>
       </c>
       <c r="B76" t="n">
@@ -1181,7 +1181,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>5_14_T514_seg0.csv</t>
+          <t>5_28_T436_seg0.csv</t>
         </is>
       </c>
       <c r="B77" t="n">
@@ -1191,7 +1191,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>5_14_T517_seg0.csv</t>
+          <t>5_28_T437_seg0.csv</t>
         </is>
       </c>
       <c r="B78" t="n">
@@ -1201,7 +1201,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>5_14_T519_seg0.csv</t>
+          <t>5_28_T439_seg0.csv</t>
         </is>
       </c>
       <c r="B79" t="n">
@@ -1211,7 +1211,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>5_28_T356_seg2.csv</t>
+          <t>5_28_T440_seg4.csv</t>
         </is>
       </c>
       <c r="B80" t="n">
@@ -1221,17 +1221,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>5_28_T358_seg13.csv</t>
+          <t>5_28_T444_seg0.csv</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>5_28_T359_seg21.csv</t>
+          <t>5_28_T447_seg0.csv</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -1241,7 +1241,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>5_28_T366_seg0.csv</t>
+          <t>5_28_T448_seg0.csv</t>
         </is>
       </c>
       <c r="B83" t="n">
@@ -1251,7 +1251,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>5_28_T372_seg0.csv</t>
+          <t>5_28_T450_seg3.csv</t>
         </is>
       </c>
       <c r="B84" t="n">
@@ -1261,7 +1261,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>5_28_T416_seg7.csv</t>
+          <t>5_28_T451_seg0.csv</t>
         </is>
       </c>
       <c r="B85" t="n">
@@ -1271,7 +1271,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>5_28_T418_seg0.csv</t>
+          <t>5_28_T452_seg0.csv</t>
         </is>
       </c>
       <c r="B86" t="n">
@@ -1281,17 +1281,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>5_28_T419_seg20.csv</t>
+          <t>5_28_T453_seg0.csv</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>5_28_T420_seg7.csv</t>
+          <t>5_28_T454_seg0.csv</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -1301,7 +1301,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>5_28_T421_seg0.csv</t>
+          <t>5_28_T455_seg4.csv</t>
         </is>
       </c>
       <c r="B89" t="n">
@@ -1311,7 +1311,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>5_28_T422_seg0.csv</t>
+          <t>5_28_T456_seg0.csv</t>
         </is>
       </c>
       <c r="B90" t="n">
@@ -1321,7 +1321,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>5_28_T423_seg0.csv</t>
+          <t>5_28_T457_seg0.csv</t>
         </is>
       </c>
       <c r="B91" t="n">
@@ -1331,7 +1331,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>5_28_T424_seg0.csv</t>
+          <t>5_28_T458_seg12.csv</t>
         </is>
       </c>
       <c r="B92" t="n">
@@ -1341,7 +1341,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>5_28_T425_seg0.csv</t>
+          <t>5_28_T460_seg0.csv</t>
         </is>
       </c>
       <c r="B93" t="n">
@@ -1351,7 +1351,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>5_28_T426_seg0.csv</t>
+          <t>5_28_T472_seg0.csv</t>
         </is>
       </c>
       <c r="B94" t="n">
@@ -1361,17 +1361,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>5_28_T427_seg0.csv</t>
+          <t>5_28_T484_seg0.csv</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>5_28_T429_seg0.csv</t>
+          <t>5_28_T487_seg0.csv</t>
         </is>
       </c>
       <c r="B96" t="n">
@@ -1381,17 +1381,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>5_28_T430_seg0.csv</t>
+          <t>5_28_T488_seg0.csv</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>5_28_T431_seg0.csv</t>
+          <t>5_28_T509_seg0.csv</t>
         </is>
       </c>
       <c r="B98" t="n">
@@ -1401,7 +1401,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>5_28_T432_seg0.csv</t>
+          <t>5_28_T512_seg0.csv</t>
         </is>
       </c>
       <c r="B99" t="n">
@@ -1411,7 +1411,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>5_28_T435_seg0.csv</t>
+          <t>5_28_T513_seg0.csv</t>
         </is>
       </c>
       <c r="B100" t="n">
@@ -1421,7 +1421,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>5_28_T436_seg0.csv</t>
+          <t>5_28_T514_seg2.csv</t>
         </is>
       </c>
       <c r="B101" t="n">
@@ -1431,7 +1431,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>5_28_T437_seg0.csv</t>
+          <t>5_28_T516_seg4.csv</t>
         </is>
       </c>
       <c r="B102" t="n">
@@ -1441,7 +1441,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>5_28_T439_seg0.csv</t>
+          <t>5_28_T517_seg0.csv</t>
         </is>
       </c>
       <c r="B103" t="n">
@@ -1451,7 +1451,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>5_28_T440_seg4.csv</t>
+          <t>5_28_T519_seg0.csv</t>
         </is>
       </c>
       <c r="B104" t="n">
@@ -1461,37 +1461,37 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>5_28_T444_seg0.csv</t>
+          <t>5_28_T520_seg0.csv</t>
         </is>
       </c>
       <c r="B105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>5_28_T445_seg0.csv</t>
+          <t>6_11_T101_seg0.csv</t>
         </is>
       </c>
       <c r="B106" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>5_28_T447_seg0.csv</t>
+          <t>6_11_T356_seg0.csv</t>
         </is>
       </c>
       <c r="B107" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>5_28_T448_seg0.csv</t>
+          <t>6_11_T358_seg0.csv</t>
         </is>
       </c>
       <c r="B108" t="n">
@@ -1501,7 +1501,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>5_28_T450_seg3.csv</t>
+          <t>6_11_T359_seg1.csv</t>
         </is>
       </c>
       <c r="B109" t="n">
@@ -1511,7 +1511,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>5_28_T451_seg0.csv</t>
+          <t>6_11_T366_seg0.csv</t>
         </is>
       </c>
       <c r="B110" t="n">
@@ -1521,7 +1521,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>5_28_T452_seg0.csv</t>
+          <t>6_11_T372_seg0.csv</t>
         </is>
       </c>
       <c r="B111" t="n">
@@ -1531,27 +1531,27 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>5_28_T453_seg0.csv</t>
+          <t>6_11_T373_seg0.csv</t>
         </is>
       </c>
       <c r="B112" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>5_28_T454_seg0.csv</t>
+          <t>6_11_T376_seg2.csv</t>
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>5_28_T455_seg4.csv</t>
+          <t>6_11_T377_seg0.csv</t>
         </is>
       </c>
       <c r="B114" t="n">
@@ -1561,7 +1561,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>5_28_T456_seg0.csv</t>
+          <t>6_11_T416_seg0.csv</t>
         </is>
       </c>
       <c r="B115" t="n">
@@ -1571,7 +1571,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>5_28_T457_seg0.csv</t>
+          <t>6_11_T418_seg0.csv</t>
         </is>
       </c>
       <c r="B116" t="n">
@@ -1581,7 +1581,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>5_28_T458_seg12.csv</t>
+          <t>6_11_T419_seg0.csv</t>
         </is>
       </c>
       <c r="B117" t="n">
@@ -1591,7 +1591,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>5_28_T460_seg0.csv</t>
+          <t>6_11_T420_seg0.csv</t>
         </is>
       </c>
       <c r="B118" t="n">
@@ -1601,7 +1601,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>5_28_T472_seg0.csv</t>
+          <t>6_11_T422_seg0.csv</t>
         </is>
       </c>
       <c r="B119" t="n">
@@ -1611,7 +1611,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>5_28_T481_seg0.csv</t>
+          <t>6_11_T423_seg24.csv</t>
         </is>
       </c>
       <c r="B120" t="n">
@@ -1621,7 +1621,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>5_28_T482_seg19.csv</t>
+          <t>6_11_T425_seg0.csv</t>
         </is>
       </c>
       <c r="B121" t="n">
@@ -1631,7 +1631,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>5_28_T483_seg0.csv</t>
+          <t>6_11_T427_seg0.csv</t>
         </is>
       </c>
       <c r="B122" t="n">
@@ -1641,7 +1641,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>5_28_T484_seg0.csv</t>
+          <t>6_11_T429_seg0.csv</t>
         </is>
       </c>
       <c r="B123" t="n">
@@ -1651,7 +1651,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>5_28_T487_seg0.csv</t>
+          <t>6_11_T430_seg0.csv</t>
         </is>
       </c>
       <c r="B124" t="n">
@@ -1661,7 +1661,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>5_28_T488_seg0.csv</t>
+          <t>6_11_T431_seg0.csv</t>
         </is>
       </c>
       <c r="B125" t="n">
@@ -1671,17 +1671,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>5_28_T503_seg0.csv</t>
+          <t>6_11_T432_seg0.csv</t>
         </is>
       </c>
       <c r="B126" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>5_28_T509_seg0.csv</t>
+          <t>6_11_T434_seg0.csv</t>
         </is>
       </c>
       <c r="B127" t="n">
@@ -1691,7 +1691,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>5_28_T511_seg0.csv</t>
+          <t>6_11_T435_seg9.csv</t>
         </is>
       </c>
       <c r="B128" t="n">
@@ -1701,37 +1701,37 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>5_28_T512_seg0.csv</t>
+          <t>6_11_T436_seg0.csv</t>
         </is>
       </c>
       <c r="B129" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>5_28_T513_seg0.csv</t>
+          <t>6_11_T437_seg1.csv</t>
         </is>
       </c>
       <c r="B130" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>5_28_T514_seg2.csv</t>
+          <t>6_11_T439_seg1.csv</t>
         </is>
       </c>
       <c r="B131" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>5_28_T516_seg4.csv</t>
+          <t>6_11_T440_seg0.csv</t>
         </is>
       </c>
       <c r="B132" t="n">
@@ -1741,7 +1741,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>5_28_T517_seg0.csv</t>
+          <t>6_11_T441_seg0.csv</t>
         </is>
       </c>
       <c r="B133" t="n">
@@ -1751,17 +1751,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>5_28_T518_seg0.csv</t>
+          <t>6_11_T442_seg0.csv</t>
         </is>
       </c>
       <c r="B134" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>5_28_T519_seg0.csv</t>
+          <t>6_11_T444_seg0.csv</t>
         </is>
       </c>
       <c r="B135" t="n">
@@ -1771,7 +1771,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>5_28_T520_seg0.csv</t>
+          <t>6_11_T448_seg0.csv</t>
         </is>
       </c>
       <c r="B136" t="n">
@@ -1781,7 +1781,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>6_11_T101_seg0.csv</t>
+          <t>6_11_T449_seg23.csv</t>
         </is>
       </c>
       <c r="B137" t="n">
@@ -1791,17 +1791,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>6_11_T356_seg0.csv</t>
+          <t>6_11_T450_seg0.csv</t>
         </is>
       </c>
       <c r="B138" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>6_11_T357_seg0.csv</t>
+          <t>6_11_T451_seg0.csv</t>
         </is>
       </c>
       <c r="B139" t="n">
@@ -1811,7 +1811,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>6_11_T358_seg0.csv</t>
+          <t>6_11_T454_seg0.csv</t>
         </is>
       </c>
       <c r="B140" t="n">
@@ -1821,7 +1821,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>6_11_T359_seg1.csv</t>
+          <t>6_11_T455_seg0.csv</t>
         </is>
       </c>
       <c r="B141" t="n">
@@ -1831,7 +1831,7 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>6_11_T366_seg0.csv</t>
+          <t>6_11_T456_seg0.csv</t>
         </is>
       </c>
       <c r="B142" t="n">
@@ -1841,7 +1841,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>6_11_T372_seg0.csv</t>
+          <t>6_11_T457_seg0.csv</t>
         </is>
       </c>
       <c r="B143" t="n">
@@ -1851,17 +1851,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>6_11_T373_seg0.csv</t>
+          <t>6_11_T460_seg0.csv</t>
         </is>
       </c>
       <c r="B144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>6_11_T376_seg2.csv</t>
+          <t>6_11_T472_seg0.csv</t>
         </is>
       </c>
       <c r="B145" t="n">
@@ -1871,7 +1871,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>6_11_T377_seg0.csv</t>
+          <t>6_11_T481_seg0.csv</t>
         </is>
       </c>
       <c r="B146" t="n">
@@ -1881,7 +1881,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>6_11_T416_seg0.csv</t>
+          <t>6_11_T482_seg0.csv</t>
         </is>
       </c>
       <c r="B147" t="n">
@@ -1891,17 +1891,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>6_11_T418_seg0.csv</t>
+          <t>6_11_T483_seg0.csv</t>
         </is>
       </c>
       <c r="B148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>6_11_T419_seg0.csv</t>
+          <t>6_11_T485_seg0.csv</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -1911,7 +1911,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>6_11_T420_seg0.csv</t>
+          <t>6_11_T487_seg0.csv</t>
         </is>
       </c>
       <c r="B150" t="n">
@@ -1921,7 +1921,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>6_11_T422_seg0.csv</t>
+          <t>6_11_T488_seg0.csv</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -1931,7 +1931,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>6_11_T423_seg24.csv</t>
+          <t>6_11_T503_seg0.csv</t>
         </is>
       </c>
       <c r="B152" t="n">
@@ -1941,7 +1941,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>6_11_T425_seg0.csv</t>
+          <t>6_11_T509_seg0.csv</t>
         </is>
       </c>
       <c r="B153" t="n">
@@ -1951,7 +1951,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>6_11_T426_seg0.csv</t>
+          <t>6_11_T511_seg0.csv</t>
         </is>
       </c>
       <c r="B154" t="n">
@@ -1961,7 +1961,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>6_11_T427_seg0.csv</t>
+          <t>6_11_T512_seg2.csv</t>
         </is>
       </c>
       <c r="B155" t="n">
@@ -1971,17 +1971,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>6_11_T428_seg0.csv</t>
+          <t>6_11_T514_seg0.csv</t>
         </is>
       </c>
       <c r="B156" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>6_11_T429_seg0.csv</t>
+          <t>6_11_T516_seg0.csv</t>
         </is>
       </c>
       <c r="B157" t="n">
@@ -1991,7 +1991,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>6_11_T430_seg0.csv</t>
+          <t>6_11_T517_seg0.csv</t>
         </is>
       </c>
       <c r="B158" t="n">
@@ -2001,7 +2001,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>6_11_T431_seg0.csv</t>
+          <t>6_11_T518_seg5.csv</t>
         </is>
       </c>
       <c r="B159" t="n">
@@ -2011,7 +2011,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>6_11_T432_seg0.csv</t>
+          <t>6_11_T519_seg0.csv</t>
         </is>
       </c>
       <c r="B160" t="n">
@@ -2021,17 +2021,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>6_11_T434_seg0.csv</t>
+          <t>6_25_T356_seg2.csv</t>
         </is>
       </c>
       <c r="B161" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>6_11_T435_seg9.csv</t>
+          <t>6_25_T357_seg0.csv</t>
         </is>
       </c>
       <c r="B162" t="n">
@@ -2041,47 +2041,47 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>6_11_T436_seg0.csv</t>
+          <t>6_25_T358_seg0.csv</t>
         </is>
       </c>
       <c r="B163" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>6_11_T437_seg1.csv</t>
+          <t>6_25_T366_seg0.csv</t>
         </is>
       </c>
       <c r="B164" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>6_11_T439_seg1.csv</t>
+          <t>6_25_T373_seg0.csv</t>
         </is>
       </c>
       <c r="B165" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>6_11_T440_seg0.csv</t>
+          <t>6_25_T376_seg21.csv</t>
         </is>
       </c>
       <c r="B166" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>6_11_T441_seg0.csv</t>
+          <t>6_25_T416_seg0.csv</t>
         </is>
       </c>
       <c r="B167" t="n">
@@ -2091,27 +2091,27 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>6_11_T442_seg0.csv</t>
+          <t>6_25_T420_seg0.csv</t>
         </is>
       </c>
       <c r="B168" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>6_11_T444_seg0.csv</t>
+          <t>6_25_T421_seg0.csv</t>
         </is>
       </c>
       <c r="B169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>6_11_T445_seg7.csv</t>
+          <t>6_25_T422_seg0.csv</t>
         </is>
       </c>
       <c r="B170" t="n">
@@ -2121,7 +2121,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>6_11_T447_seg0.csv</t>
+          <t>6_25_T423_seg6.csv</t>
         </is>
       </c>
       <c r="B171" t="n">
@@ -2131,7 +2131,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>6_11_T448_seg0.csv</t>
+          <t>6_25_T424_seg0.csv</t>
         </is>
       </c>
       <c r="B172" t="n">
@@ -2141,7 +2141,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>6_11_T449_seg23.csv</t>
+          <t>6_25_T425_seg0.csv</t>
         </is>
       </c>
       <c r="B173" t="n">
@@ -2151,7 +2151,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>6_11_T450_seg0.csv</t>
+          <t>6_25_T432_seg0.csv</t>
         </is>
       </c>
       <c r="B174" t="n">
@@ -2161,17 +2161,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>6_11_T451_seg0.csv</t>
+          <t>6_25_T434_seg0.csv</t>
         </is>
       </c>
       <c r="B175" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>6_11_T454_seg0.csv</t>
+          <t>6_25_T435_seg0.csv</t>
         </is>
       </c>
       <c r="B176" t="n">
@@ -2181,17 +2181,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>6_11_T455_seg0.csv</t>
+          <t>6_25_T436_seg13.csv</t>
         </is>
       </c>
       <c r="B177" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>6_11_T456_seg0.csv</t>
+          <t>6_25_T442_seg0.csv</t>
         </is>
       </c>
       <c r="B178" t="n">
@@ -2201,7 +2201,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>6_11_T457_seg0.csv</t>
+          <t>6_25_T445_seg0.csv</t>
         </is>
       </c>
       <c r="B179" t="n">
@@ -2211,7 +2211,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>6_11_T458_seg0.csv</t>
+          <t>6_25_T447_seg11.csv</t>
         </is>
       </c>
       <c r="B180" t="n">
@@ -2221,17 +2221,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>6_11_T459_seg2.csv</t>
+          <t>6_25_T448_seg5.csv</t>
         </is>
       </c>
       <c r="B181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>6_11_T460_seg0.csv</t>
+          <t>6_25_T449_seg0.csv</t>
         </is>
       </c>
       <c r="B182" t="n">
@@ -2241,7 +2241,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>6_11_T472_seg0.csv</t>
+          <t>6_25_T450_seg1.csv</t>
         </is>
       </c>
       <c r="B183" t="n">
@@ -2251,7 +2251,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>6_11_T481_seg0.csv</t>
+          <t>6_25_T451_seg0.csv</t>
         </is>
       </c>
       <c r="B184" t="n">
@@ -2261,7 +2261,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>6_11_T482_seg0.csv</t>
+          <t>6_25_T452_seg0.csv</t>
         </is>
       </c>
       <c r="B185" t="n">
@@ -2271,17 +2271,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>6_11_T483_seg0.csv</t>
+          <t>6_25_T454_seg0.csv</t>
         </is>
       </c>
       <c r="B186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>6_11_T484_seg3.csv</t>
+          <t>6_25_T455_seg0.csv</t>
         </is>
       </c>
       <c r="B187" t="n">
@@ -2291,7 +2291,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>6_11_T485_seg0.csv</t>
+          <t>6_25_T458_seg0.csv</t>
         </is>
       </c>
       <c r="B188" t="n">
@@ -2301,7 +2301,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>6_11_T486_seg0.csv</t>
+          <t>6_25_T459_seg0.csv</t>
         </is>
       </c>
       <c r="B189" t="n">
@@ -2311,17 +2311,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>6_11_T487_seg0.csv</t>
+          <t>6_25_T460_seg3.csv</t>
         </is>
       </c>
       <c r="B190" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>6_11_T488_seg0.csv</t>
+          <t>6_25_T472_seg0.csv</t>
         </is>
       </c>
       <c r="B191" t="n">
@@ -2331,7 +2331,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>6_11_T503_seg0.csv</t>
+          <t>6_25_T481_seg0.csv</t>
         </is>
       </c>
       <c r="B192" t="n">
@@ -2341,7 +2341,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>6_11_T509_seg0.csv</t>
+          <t>6_25_T483_seg0.csv</t>
         </is>
       </c>
       <c r="B193" t="n">
@@ -2351,17 +2351,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>6_11_T511_seg0.csv</t>
+          <t>6_25_T484_seg0.csv</t>
         </is>
       </c>
       <c r="B194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>6_11_T512_seg2.csv</t>
+          <t>6_25_T486_seg0.csv</t>
         </is>
       </c>
       <c r="B195" t="n">
@@ -2371,7 +2371,7 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>6_11_T513_seg0.csv</t>
+          <t>6_25_T488_seg0.csv</t>
         </is>
       </c>
       <c r="B196" t="n">
@@ -2381,7 +2381,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>6_11_T514_seg0.csv</t>
+          <t>6_25_T503_seg0.csv</t>
         </is>
       </c>
       <c r="B197" t="n">
@@ -2391,7 +2391,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>6_11_T516_seg0.csv</t>
+          <t>6_25_T509_seg15.csv</t>
         </is>
       </c>
       <c r="B198" t="n">
@@ -2401,7 +2401,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>6_11_T517_seg0.csv</t>
+          <t>6_25_T511_seg0.csv</t>
         </is>
       </c>
       <c r="B199" t="n">
@@ -2411,7 +2411,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>6_11_T518_seg5.csv</t>
+          <t>6_25_T517_seg0.csv</t>
         </is>
       </c>
       <c r="B200" t="n">
@@ -2421,7 +2421,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>6_11_T519_seg0.csv</t>
+          <t>6_25_T519_seg0.csv</t>
         </is>
       </c>
       <c r="B201" t="n">
@@ -2431,17 +2431,17 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>6_25_T356_seg2.csv</t>
+          <t>6_25_T520_seg0.csv</t>
         </is>
       </c>
       <c r="B202" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>6_25_T357_seg0.csv</t>
+          <t>6_25_Y101_seg0.csv</t>
         </is>
       </c>
       <c r="B203" t="n">
@@ -2451,7 +2451,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>6_25_T358_seg0.csv</t>
+          <t>7_10_458_seg0.csv</t>
         </is>
       </c>
       <c r="B204" t="n">
@@ -2461,17 +2461,17 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>6_25_T359_seg0.csv</t>
+          <t>7_10_460_seg4.csv</t>
         </is>
       </c>
       <c r="B205" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>6_25_T366_seg0.csv</t>
+          <t>7_10_482_seg0.csv</t>
         </is>
       </c>
       <c r="B206" t="n">
@@ -2481,7 +2481,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>6_25_T373_seg0.csv</t>
+          <t>7_10_483_seg5.csv</t>
         </is>
       </c>
       <c r="B207" t="n">
@@ -2491,17 +2491,17 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>6_25_T376_seg21.csv</t>
+          <t>7_10_488_seg0.csv</t>
         </is>
       </c>
       <c r="B208" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>6_25_T377_seg9.csv</t>
+          <t>7_10_517_seg0.csv</t>
         </is>
       </c>
       <c r="B209" t="n">
@@ -2511,7 +2511,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>6_25_T416_seg0.csv</t>
+          <t>7_10_519_seg23.csv</t>
         </is>
       </c>
       <c r="B210" t="n">
@@ -2521,7 +2521,7 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>6_25_T420_seg0.csv</t>
+          <t>7_10_520_seg0.csv</t>
         </is>
       </c>
       <c r="B211" t="n">
@@ -2531,17 +2531,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>6_25_T421_seg0.csv</t>
+          <t>7_10_T356_seg24.csv</t>
         </is>
       </c>
       <c r="B212" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>6_25_T422_seg0.csv</t>
+          <t>7_10_T357_seg0.csv</t>
         </is>
       </c>
       <c r="B213" t="n">
@@ -2551,7 +2551,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>6_25_T423_seg6.csv</t>
+          <t>7_10_T359_seg0.csv</t>
         </is>
       </c>
       <c r="B214" t="n">
@@ -2561,7 +2561,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>6_25_T424_seg0.csv</t>
+          <t>7_10_T372_seg0.csv</t>
         </is>
       </c>
       <c r="B215" t="n">
@@ -2571,37 +2571,37 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>6_25_T425_seg0.csv</t>
+          <t>7_10_T373_seg0.csv</t>
         </is>
       </c>
       <c r="B216" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>6_25_T432_seg0.csv</t>
+          <t>7_10_T376_seg0.csv</t>
         </is>
       </c>
       <c r="B217" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>6_25_T434_seg0.csv</t>
+          <t>7_10_T377_seg0.csv</t>
         </is>
       </c>
       <c r="B218" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>6_25_T435_seg0.csv</t>
+          <t>7_10_T416_seg0.csv</t>
         </is>
       </c>
       <c r="B219" t="n">
@@ -2611,17 +2611,17 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>6_25_T436_seg13.csv</t>
+          <t>7_10_T418_seg1.csv</t>
         </is>
       </c>
       <c r="B220" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>6_25_T437_seg1.csv</t>
+          <t>7_10_T419_seg0.csv</t>
         </is>
       </c>
       <c r="B221" t="n">
@@ -2631,7 +2631,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>6_25_T439_seg0.csv</t>
+          <t>7_10_T420_seg0.csv</t>
         </is>
       </c>
       <c r="B222" t="n">
@@ -2641,7 +2641,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>6_25_T442_seg0.csv</t>
+          <t>7_10_T421_seg0.csv</t>
         </is>
       </c>
       <c r="B223" t="n">
@@ -2651,7 +2651,7 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>6_25_T445_seg0.csv</t>
+          <t>7_10_T422_seg0.csv</t>
         </is>
       </c>
       <c r="B224" t="n">
@@ -2661,7 +2661,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>6_25_T447_seg11.csv</t>
+          <t>7_10_T423_seg0.csv</t>
         </is>
       </c>
       <c r="B225" t="n">
@@ -2671,17 +2671,17 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>6_25_T448_seg5.csv</t>
+          <t>7_10_T426_seg0.csv</t>
         </is>
       </c>
       <c r="B226" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>6_25_T449_seg0.csv</t>
+          <t>7_10_T427_seg0.csv</t>
         </is>
       </c>
       <c r="B227" t="n">
@@ -2691,17 +2691,17 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>6_25_T450_seg1.csv</t>
+          <t>7_10_T428_seg0.csv</t>
         </is>
       </c>
       <c r="B228" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>6_25_T451_seg0.csv</t>
+          <t>7_10_T429_seg0.csv</t>
         </is>
       </c>
       <c r="B229" t="n">
@@ -2711,7 +2711,7 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>6_25_T452_seg0.csv</t>
+          <t>7_10_T430_seg0.csv</t>
         </is>
       </c>
       <c r="B230" t="n">
@@ -2721,7 +2721,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>6_25_T454_seg0.csv</t>
+          <t>7_10_T434_seg0.csv</t>
         </is>
       </c>
       <c r="B231" t="n">
@@ -2731,7 +2731,7 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>6_25_T455_seg0.csv</t>
+          <t>7_10_T435_seg0.csv</t>
         </is>
       </c>
       <c r="B232" t="n">
@@ -2741,7 +2741,7 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>6_25_T457_seg0.csv</t>
+          <t>7_10_T436_seg0.csv</t>
         </is>
       </c>
       <c r="B233" t="n">
@@ -2751,17 +2751,17 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>6_25_T458_seg0.csv</t>
+          <t>7_10_T437_seg0.csv</t>
         </is>
       </c>
       <c r="B234" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>6_25_T459_seg0.csv</t>
+          <t>7_10_T439_seg0.csv</t>
         </is>
       </c>
       <c r="B235" t="n">
@@ -2771,7 +2771,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>6_25_T460_seg3.csv</t>
+          <t>7_10_T440_seg1.csv</t>
         </is>
       </c>
       <c r="B236" t="n">
@@ -2781,37 +2781,37 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>6_25_T472_seg0.csv</t>
+          <t>7_10_T442_seg1.csv</t>
         </is>
       </c>
       <c r="B237" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>6_25_T481_seg0.csv</t>
+          <t>7_10_T443_seg0.csv</t>
         </is>
       </c>
       <c r="B238" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>6_25_T483_seg0.csv</t>
+          <t>7_10_T444_seg0.csv</t>
         </is>
       </c>
       <c r="B239" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>6_25_T484_seg0.csv</t>
+          <t>7_10_T447_seg11.csv</t>
         </is>
       </c>
       <c r="B240" t="n">
@@ -2821,7 +2821,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>6_25_T486_seg0.csv</t>
+          <t>7_10_T448_seg0.csv</t>
         </is>
       </c>
       <c r="B241" t="n">
@@ -2831,17 +2831,17 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>6_25_T488_seg0.csv</t>
+          <t>7_10_T449_seg0.csv</t>
         </is>
       </c>
       <c r="B242" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>6_25_T503_seg0.csv</t>
+          <t>7_10_T450_seg0.csv</t>
         </is>
       </c>
       <c r="B243" t="n">
@@ -2851,7 +2851,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>6_25_T509_seg15.csv</t>
+          <t>7_10_T452_seg0.csv</t>
         </is>
       </c>
       <c r="B244" t="n">
@@ -2861,7 +2861,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>6_25_T511_seg0.csv</t>
+          <t>7_10_T454_seg15.csv</t>
         </is>
       </c>
       <c r="B245" t="n">
@@ -2871,7 +2871,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>6_25_T512_seg0.csv</t>
+          <t>7_10_T455_seg0.csv</t>
         </is>
       </c>
       <c r="B246" t="n">
@@ -2881,7 +2881,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>6_25_T517_seg0.csv</t>
+          <t>7_10_T456_seg0.csv</t>
         </is>
       </c>
       <c r="B247" t="n">
@@ -2891,7 +2891,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>6_25_T519_seg0.csv</t>
+          <t>7_10_T457_seg2.csv</t>
         </is>
       </c>
       <c r="B248" t="n">
@@ -2901,7 +2901,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>6_25_T520_seg0.csv</t>
+          <t>7_10_T472_seg0.csv</t>
         </is>
       </c>
       <c r="B249" t="n">
@@ -2911,7 +2911,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>6_25_Y101_seg0.csv</t>
+          <t>7_10_T482_seg11.csv</t>
         </is>
       </c>
       <c r="B250" t="n">
@@ -2921,7 +2921,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>7_10_458_seg0.csv</t>
+          <t>7_10_T486_seg0.csv</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -2931,7 +2931,7 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>7_10_459_seg0.csv</t>
+          <t>7_10_T487_seg0.csv</t>
         </is>
       </c>
       <c r="B252" t="n">
@@ -2941,17 +2941,17 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>7_10_460_seg4.csv</t>
+          <t>7_10_T511_seg0.csv</t>
         </is>
       </c>
       <c r="B253" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>7_10_482_seg0.csv</t>
+          <t>7_10_T512_seg0.csv</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -2961,7 +2961,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>7_10_483_seg5.csv</t>
+          <t>7_10_T514_seg0.csv</t>
         </is>
       </c>
       <c r="B255" t="n">
@@ -2971,610 +2971,10 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>7_10_484_seg1.csv</t>
+          <t>7_10_T516_seg0.csv</t>
         </is>
       </c>
       <c r="B256" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>7_10_488_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B257" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>7_10_517_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B258" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>7_10_519_seg23.csv</t>
-        </is>
-      </c>
-      <c r="B259" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>7_10_520_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B260" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>7_10_T356_seg24.csv</t>
-        </is>
-      </c>
-      <c r="B261" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>7_10_T357_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B262" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>7_10_T358_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B263" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>7_10_T359_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B264" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>7_10_T366_seg28.csv</t>
-        </is>
-      </c>
-      <c r="B265" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>7_10_T372_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B266" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
-          <t>7_10_T373_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B267" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>7_10_T376_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B268" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>7_10_T377_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B269" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>7_10_T416_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B270" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>7_10_T418_seg1.csv</t>
-        </is>
-      </c>
-      <c r="B271" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>7_10_T419_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B272" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>7_10_T420_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B273" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>7_10_T421_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B274" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>7_10_T422_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B275" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>7_10_T423_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B276" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>7_10_T424_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B277" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>7_10_T426_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B278" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>7_10_T427_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B279" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>7_10_T428_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B280" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>7_10_T429_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B281" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
-        <is>
-          <t>7_10_T430_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B282" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
-        <is>
-          <t>7_10_T431_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B283" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
-        <is>
-          <t>7_10_T432_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B284" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
-        <is>
-          <t>7_10_T434_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B285" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
-        <is>
-          <t>7_10_T435_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B286" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t>7_10_T436_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B287" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>7_10_T437_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B288" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t>7_10_T439_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B289" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>7_10_T440_seg1.csv</t>
-        </is>
-      </c>
-      <c r="B290" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>7_10_T442_seg1.csv</t>
-        </is>
-      </c>
-      <c r="B291" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>7_10_T443_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B292" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>7_10_T444_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B293" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>7_10_T445_seg1.csv</t>
-        </is>
-      </c>
-      <c r="B294" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>7_10_T447_seg11.csv</t>
-        </is>
-      </c>
-      <c r="B295" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="296">
-      <c r="A296" t="inlineStr">
-        <is>
-          <t>7_10_T448_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B296" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="297">
-      <c r="A297" t="inlineStr">
-        <is>
-          <t>7_10_T449_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B297" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="298">
-      <c r="A298" t="inlineStr">
-        <is>
-          <t>7_10_T450_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B298" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="299">
-      <c r="A299" t="inlineStr">
-        <is>
-          <t>7_10_T451_seg7.csv</t>
-        </is>
-      </c>
-      <c r="B299" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="300">
-      <c r="A300" t="inlineStr">
-        <is>
-          <t>7_10_T452_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B300" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="301">
-      <c r="A301" t="inlineStr">
-        <is>
-          <t>7_10_T454_seg15.csv</t>
-        </is>
-      </c>
-      <c r="B301" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" t="inlineStr">
-        <is>
-          <t>7_10_T455_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B302" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="303">
-      <c r="A303" t="inlineStr">
-        <is>
-          <t>7_10_T456_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B303" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="304">
-      <c r="A304" t="inlineStr">
-        <is>
-          <t>7_10_T457_seg2.csv</t>
-        </is>
-      </c>
-      <c r="B304" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="305">
-      <c r="A305" t="inlineStr">
-        <is>
-          <t>7_10_T472_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B305" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="306">
-      <c r="A306" t="inlineStr">
-        <is>
-          <t>7_10_T482_seg11.csv</t>
-        </is>
-      </c>
-      <c r="B306" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="307">
-      <c r="A307" t="inlineStr">
-        <is>
-          <t>7_10_T485_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B307" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="308">
-      <c r="A308" t="inlineStr">
-        <is>
-          <t>7_10_T486_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B308" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="309">
-      <c r="A309" t="inlineStr">
-        <is>
-          <t>7_10_T487_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B309" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="310">
-      <c r="A310" t="inlineStr">
-        <is>
-          <t>7_10_T503_seg7.csv</t>
-        </is>
-      </c>
-      <c r="B310" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="311">
-      <c r="A311" t="inlineStr">
-        <is>
-          <t>7_10_T509_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B311" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="312">
-      <c r="A312" t="inlineStr">
-        <is>
-          <t>7_10_T511_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B312" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>7_10_T512_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B313" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="314">
-      <c r="A314" t="inlineStr">
-        <is>
-          <t>7_10_T514_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B314" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="315">
-      <c r="A315" t="inlineStr">
-        <is>
-          <t>7_10_T516_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B315" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="316">
-      <c r="A316" t="inlineStr">
-        <is>
-          <t>7_10_Y101_seg0.csv</t>
-        </is>
-      </c>
-      <c r="B316" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>